<commit_message>
Implement Sprint 2.1 account shell fixes
</commit_message>
<xml_diff>
--- a/acceptance_matrix.xlsx
+++ b/acceptance_matrix.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="1" r:id="R26a23ca8bdf84be9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Summary" sheetId="2" r:id="R5eb59a6c0bd94122"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Personas" sheetId="3" r:id="R2937e88ab87941a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Traceability" sheetId="4" r:id="R262d966e406948c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="1" r:id="R249f9a797fa943ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Summary" sheetId="2" r:id="Re0ad5a5fdbe749d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Personas" sheetId="3" r:id="Rd6e8cce3459042d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Traceability" sheetId="4" r:id="Redee6ed63b0c464c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8042,10 +8042,10 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O157" s="15" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="P157" s="15" t="str">
-        <x:v>Owner manual browser QA required after deployment — 2026-09-10</x:v>
+        <x:v>Owner manual production acceptance PASS — 2026-09-13</x:v>
       </x:c>
     </x:row>
     <x:row r="158">
@@ -8092,10 +8092,10 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O158" s="15" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="P158" s="15" t="str">
-        <x:v>Owner manual browser QA required after deployment — 2026-09-10</x:v>
+        <x:v>Owner manual production acceptance PASS — 2026-09-13</x:v>
       </x:c>
     </x:row>
     <x:row r="159">
@@ -8692,9 +8692,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O170" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P170" s="15" t="str"/>
+        <x:v>Fail</x:v>
+      </x:c>
+      <x:c r="P170" s="15" t="str">
+        <x:v>Owner production acceptance FAIL — 2026-09-13: Store Owner account area requires the Sprint 2.1 dashboard/navigation fix and owner retest.</x:v>
+      </x:c>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="15" t="str">
@@ -17409,7 +17411,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda49dbaba0a24b9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e6969bc02de49e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17579,7 +17581,7 @@
       </x:c>
       <x:c r="B10" s="12" t="n">
         <x:f>COUNTIF('Acceptance Matrix'!O2:O350,"Pass")</x:f>
-        <x:v>78</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
         <x:v>Stores</x:v>
@@ -17599,7 +17601,7 @@
       </x:c>
       <x:c r="B11" s="12" t="n">
         <x:f>COUNTIF('Acceptance Matrix'!O2:O350,"Fail")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
         <x:v>Store Dashboard</x:v>
@@ -17946,7 +17948,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fb3748f2e1146e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a6b794493974eaf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18286,7 +18288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaf06f0db1c748e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82f2f46a36c942b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implement Sprint 3 listing lifecycle and revisions
</commit_message>
<xml_diff>
--- a/acceptance_matrix.xlsx
+++ b/acceptance_matrix.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="1" r:id="R249f9a797fa943ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Summary" sheetId="2" r:id="Re0ad5a5fdbe749d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Personas" sheetId="3" r:id="Rd6e8cce3459042d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Traceability" sheetId="4" r:id="Redee6ed63b0c464c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="1" r:id="R8939972c58b54712"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Summary" sheetId="2" r:id="Rf7ff0b70ad76432f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Personas" sheetId="3" r:id="Rfb4b745ffbd64de2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Traceability" sheetId="4" r:id="Ra0c418e7fad74fff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8692,10 +8692,10 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O170" s="15" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="P170" s="15" t="str">
-        <x:v>Owner production acceptance FAIL — 2026-09-13: Store Owner account area requires the Sprint 2.1 dashboard/navigation fix and owner retest.</x:v>
+        <x:v>Owner manual production retest PASS — 2026-09-13</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -17411,7 +17411,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e6969bc02de49e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra74909d83f4d43f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17581,7 +17581,7 @@
       </x:c>
       <x:c r="B10" s="12" t="n">
         <x:f>COUNTIF('Acceptance Matrix'!O2:O350,"Pass")</x:f>
-        <x:v>80</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
         <x:v>Stores</x:v>
@@ -17601,7 +17601,7 @@
       </x:c>
       <x:c r="B11" s="12" t="n">
         <x:f>COUNTIF('Acceptance Matrix'!O2:O350,"Fail")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
         <x:v>Store Dashboard</x:v>
@@ -17948,7 +17948,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a6b794493974eaf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99960cbd21274bf4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18288,7 +18288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82f2f46a36c942b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R068000dbfd654911"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Sprint 3 acceptance and add amendable revisions and notifications
</commit_message>
<xml_diff>
--- a/acceptance_matrix.xlsx
+++ b/acceptance_matrix.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="1" r:id="R8939972c58b54712"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Summary" sheetId="2" r:id="Rf7ff0b70ad76432f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Personas" sheetId="3" r:id="Rfb4b745ffbd64de2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Traceability" sheetId="4" r:id="Ra0c418e7fad74fff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="1" r:id="R46927f09d30a493e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Summary" sheetId="2" r:id="R22def8a16b854d9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Personas" sheetId="3" r:id="Rec6f6c5a61be4896"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Traceability" sheetId="4" r:id="R550ac3b380bc45d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AcceptanceMatrix" displayName="AcceptanceMatrix" ref="A1:P350" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AcceptanceMatrix" displayName="AcceptanceMatrix" ref="A1:P358" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Domain"/>
@@ -2490,9 +2490,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O43" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P43" s="15" t="str"/>
+        <x:v>Fail</x:v>
+      </x:c>
+      <x:c r="P43" s="15" t="str">
+        <x:v>Owner production acceptance FAIL — S/ 1,200 rendered as S/ 1,197 — 2026-09-15; fix awaits owner retest.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="15" t="str">
@@ -4482,9 +4484,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O84" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P84" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P84" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="15" t="str">
@@ -4530,9 +4534,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O85" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P85" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P85" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="15" t="str">
@@ -4578,9 +4584,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O86" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P86" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P86" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="15" t="str">
@@ -4626,9 +4634,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O87" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P87" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P87" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="15" t="str">
@@ -4770,9 +4780,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O90" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P90" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P90" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="15" t="str">
@@ -4962,9 +4974,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O94" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P94" s="15" t="str"/>
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="P94" s="15" t="str">
+        <x:v>Deferred — requires the later verified-transaction/review system.</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="15" t="str">
@@ -5010,9 +5024,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O95" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P95" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P95" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="15" t="str">
@@ -5250,9 +5266,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O100" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P100" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P100" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="15" t="str">
@@ -5490,9 +5508,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O105" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P105" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P105" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="15" t="str">
@@ -5538,9 +5558,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O106" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P106" s="15" t="str"/>
+        <x:v>Fail</x:v>
+      </x:c>
+      <x:c r="P106" s="15" t="str">
+        <x:v>Owner production acceptance FAIL — mixed moderated/photo edit returned an action error — 2026-09-15; fix awaits owner retest.</x:v>
+      </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="15" t="str">
@@ -5586,9 +5608,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O107" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P107" s="15" t="str"/>
+        <x:v>Fail</x:v>
+      </x:c>
+      <x:c r="P107" s="15" t="str">
+        <x:v>Owner production acceptance FAIL — approved title was not the primary public title — 2026-09-15; fix awaits owner retest.</x:v>
+      </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="15" t="str">
@@ -5634,9 +5658,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O108" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P108" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P108" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="15" t="str">
@@ -5649,16 +5675,16 @@
         <x:v>Approved listing revisions</x:v>
       </x:c>
       <x:c r="D109" s="15" t="str">
-        <x:v>Second moderated edit while revision pending is safely handled</x:v>
+        <x:v>Additional moderated edits safely amend the existing pending proposal</x:v>
       </x:c>
       <x:c r="E109" s="15" t="str">
-        <x:v>Pending revision exists.</x:v>
+        <x:v>Approved listing with one pending moderated revision.</x:v>
       </x:c>
       <x:c r="F109" s="15" t="str">
-        <x:v>Owner attempts another moderated edit.</x:v>
+        <x:v>Change another moderated field or the proposed photos before the admin decision.</x:v>
       </x:c>
       <x:c r="G109" s="15" t="str">
-        <x:v>System follows defined safe behavior without overwriting live approved state or losing revision history.</x:v>
+        <x:v>Exactly one pending revision remains and contains the latest complete proposed moderated state.</x:v>
       </x:c>
       <x:c r="H109" s="15" t="str">
         <x:v>Particular</x:v>
@@ -5682,9 +5708,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O109" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P109" s="15" t="str"/>
+        <x:v>Fail</x:v>
+      </x:c>
+      <x:c r="P109" s="15" t="str">
+        <x:v>Requirement updated for amendable pending proposals; implementation awaits owner production retest — 2026-09-16.</x:v>
+      </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="15" t="str">
@@ -5730,9 +5758,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O110" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P110" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P110" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="15" t="str">
@@ -5778,9 +5808,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O111" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P111" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P111" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="15" t="str">
@@ -5826,9 +5858,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O112" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P112" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P112" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="15" t="str">
@@ -5874,9 +5908,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O113" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P113" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P113" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="15" t="str">
@@ -5922,9 +5958,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O114" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P114" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P114" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="15" t="str">
@@ -5970,9 +6008,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O115" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P115" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P115" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="15" t="str">
@@ -6018,9 +6058,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O116" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P116" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P116" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="15" t="str">
@@ -6066,9 +6108,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O117" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P117" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P117" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="15" t="str">
@@ -6114,9 +6158,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O118" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P118" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P118" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="15" t="str">
@@ -8838,9 +8884,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O173" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P173" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P173" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="15" t="str">
@@ -8886,9 +8934,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O174" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P174" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P174" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="15" t="str">
@@ -8934,9 +8984,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O175" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P175" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P175" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="15" t="str">
@@ -8982,9 +9034,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O176" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P176" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P176" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="15" t="str">
@@ -9126,9 +9180,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O179" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P179" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P179" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="15" t="str">
@@ -14840,9 +14896,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O298" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P298" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P298" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="299">
       <x:c r="A299" s="15" t="str">
@@ -15082,9 +15140,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O303" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P303" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P303" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="304">
       <x:c r="A304" s="15" t="str">
@@ -15130,9 +15190,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O304" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P304" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P304" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="305">
       <x:c r="A305" s="15" t="str">
@@ -15178,9 +15240,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O305" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P305" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P305" s="15" t="str">
+        <x:v>Owner manual production acceptance PASS — 2026-09-15</x:v>
+      </x:c>
     </x:row>
     <x:row r="306">
       <x:c r="A306" s="15" t="str">
@@ -17377,6 +17441,406 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="P350" s="15" t="str"/>
+    </x:row>
+    <x:row r="351">
+      <x:c r="A351" t="str">
+        <x:v>REV-017</x:v>
+      </x:c>
+      <x:c r="B351" t="str">
+        <x:v>Listings</x:v>
+      </x:c>
+      <x:c r="C351" t="str">
+        <x:v>Approved listing editing</x:v>
+      </x:c>
+      <x:c r="D351" t="str">
+        <x:v>Pending moderated revision is amended in place</x:v>
+      </x:c>
+      <x:c r="E351" t="str">
+        <x:v>Approved listing has a pending title proposal.</x:v>
+      </x:c>
+      <x:c r="F351" t="str">
+        <x:v>Change the proposed title again and add a moderated condition change.</x:v>
+      </x:c>
+      <x:c r="G351" t="str">
+        <x:v>The same pending revision ID is retained, its version increases, and it contains the latest proposal.</x:v>
+      </x:c>
+      <x:c r="H351" t="str">
+        <x:v>Particular</x:v>
+      </x:c>
+      <x:c r="I351" t="str">
+        <x:v>DB/Integration</x:v>
+      </x:c>
+      <x:c r="J351" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K351" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L351" t="str">
+        <x:v>Blocking</x:v>
+      </x:c>
+      <x:c r="M351" t="str">
+        <x:v>L117-L137</x:v>
+      </x:c>
+      <x:c r="N351" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="O351" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P351" t="str">
+        <x:v>Automated local Sprint 3.1 regression PASS — 2026-09-16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="352">
+      <x:c r="A352" t="str">
+        <x:v>REV-018</x:v>
+      </x:c>
+      <x:c r="B352" t="str">
+        <x:v>Listings</x:v>
+      </x:c>
+      <x:c r="C352" t="str">
+        <x:v>Approved listing editing</x:v>
+      </x:c>
+      <x:c r="D352" t="str">
+        <x:v>Pending revision photo set can be amended</x:v>
+      </x:c>
+      <x:c r="E352" t="str">
+        <x:v>Approved listing has a pending moderated proposal and valid live photos.</x:v>
+      </x:c>
+      <x:c r="F352" t="str">
+        <x:v>Add, remove, reorder or replace proposed photos and save.</x:v>
+      </x:c>
+      <x:c r="G352" t="str">
+        <x:v>The same pending proposal contains the latest isolated photo set; live photos remain unchanged until approval.</x:v>
+      </x:c>
+      <x:c r="H352" t="str">
+        <x:v>Particular</x:v>
+      </x:c>
+      <x:c r="I352" t="str">
+        <x:v>DB/Integration</x:v>
+      </x:c>
+      <x:c r="J352" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K352" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L352" t="str">
+        <x:v>Blocking</x:v>
+      </x:c>
+      <x:c r="M352" t="str">
+        <x:v>L117-L137</x:v>
+      </x:c>
+      <x:c r="N352" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="O352" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P352" t="str">
+        <x:v>Automated local Sprint 3.1 regression PASS — 2026-09-16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="353">
+      <x:c r="A353" t="str">
+        <x:v>REV-019</x:v>
+      </x:c>
+      <x:c r="B353" t="str">
+        <x:v>Listings</x:v>
+      </x:c>
+      <x:c r="C353" t="str">
+        <x:v>Approved listing editing</x:v>
+      </x:c>
+      <x:c r="D353" t="str">
+        <x:v>Stale admin revision decision is denied</x:v>
+      </x:c>
+      <x:c r="E353" t="str">
+        <x:v>Admin loaded revision version N; owner amends it to N+1.</x:v>
+      </x:c>
+      <x:c r="F353" t="str">
+        <x:v>Admin attempts approval or rejection using version N.</x:v>
+      </x:c>
+      <x:c r="G353" t="str">
+        <x:v>The decision fails safely and admin must reload the latest proposal.</x:v>
+      </x:c>
+      <x:c r="H353" t="str">
+        <x:v>Admin</x:v>
+      </x:c>
+      <x:c r="I353" t="str">
+        <x:v>DB/Integration</x:v>
+      </x:c>
+      <x:c r="J353" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K353" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L353" t="str">
+        <x:v>Blocking</x:v>
+      </x:c>
+      <x:c r="M353" t="str">
+        <x:v>L117-L137</x:v>
+      </x:c>
+      <x:c r="N353" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="O353" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P353" t="str">
+        <x:v>Automated local Sprint 3.1 regression PASS — 2026-09-16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="354">
+      <x:c r="A354" t="str">
+        <x:v>LIST-023</x:v>
+      </x:c>
+      <x:c r="B354" t="str">
+        <x:v>Listings</x:v>
+      </x:c>
+      <x:c r="C354" t="str">
+        <x:v>Particular listing creation</x:v>
+      </x:c>
+      <x:c r="D354" t="str">
+        <x:v>Whole-sol price round-trips exactly</x:v>
+      </x:c>
+      <x:c r="E354" t="str">
+        <x:v>Seller enters a valid price such as S/ 1,200.</x:v>
+      </x:c>
+      <x:c r="F354" t="str">
+        <x:v>Submit, query stored/API value, then open catalog card and detail page; repeat after price edit.</x:v>
+      </x:c>
+      <x:c r="G354" t="str">
+        <x:v>Entered, stored, API and rendered values remain exactly S/ 1,200, with no fee or numeric-control mutation.</x:v>
+      </x:c>
+      <x:c r="H354" t="str">
+        <x:v>Particular</x:v>
+      </x:c>
+      <x:c r="I354" t="str">
+        <x:v>Integration</x:v>
+      </x:c>
+      <x:c r="J354" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K354" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L354" t="str">
+        <x:v>Blocking</x:v>
+      </x:c>
+      <x:c r="M354" t="str">
+        <x:v>L59-L79</x:v>
+      </x:c>
+      <x:c r="N354" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="O354" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P354" t="str">
+        <x:v>Automated local Sprint 3.1 regression PASS — 2026-09-16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="355">
+      <x:c r="A355" t="str">
+        <x:v>STORE-018</x:v>
+      </x:c>
+      <x:c r="B355" t="str">
+        <x:v>Stores</x:v>
+      </x:c>
+      <x:c r="C355" t="str">
+        <x:v>Application and ownership</x:v>
+      </x:c>
+      <x:c r="D355" t="str">
+        <x:v>Duplicate RUC shows an explicit private reason</x:v>
+      </x:c>
+      <x:c r="E355" t="str">
+        <x:v>Another store already owns the normalized RUC.</x:v>
+      </x:c>
+      <x:c r="F355" t="str">
+        <x:v>Submit the duplicate RUC through the store application.</x:v>
+      </x:c>
+      <x:c r="G355" t="str">
+        <x:v>Submission is blocked and UI states that the RUC is already registered without exposing owner data.</x:v>
+      </x:c>
+      <x:c r="H355" t="str">
+        <x:v>Store Owner</x:v>
+      </x:c>
+      <x:c r="I355" t="str">
+        <x:v>Integration</x:v>
+      </x:c>
+      <x:c r="J355" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K355" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L355" t="str">
+        <x:v>Blocking</x:v>
+      </x:c>
+      <x:c r="M355" t="str">
+        <x:v>L139-L154</x:v>
+      </x:c>
+      <x:c r="N355" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="O355" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P355" t="str">
+        <x:v>Automated local Sprint 3.1 regression PASS — 2026-09-16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="356">
+      <x:c r="A356" t="str">
+        <x:v>DASH-008</x:v>
+      </x:c>
+      <x:c r="B356" t="str">
+        <x:v>Particular Dashboard</x:v>
+      </x:c>
+      <x:c r="C356" t="str">
+        <x:v>Account result notices</x:v>
+      </x:c>
+      <x:c r="D356" t="str">
+        <x:v>Page-level action notice receives focus and is scrolled into view</x:v>
+      </x:c>
+      <x:c r="E356" t="str">
+        <x:v>Account/admin form returns a top-level success or actionable error.</x:v>
+      </x:c>
+      <x:c r="F356" t="str">
+        <x:v>Complete the form while its notice location is outside the viewport.</x:v>
+      </x:c>
+      <x:c r="G356" t="str">
+        <x:v>The shared notice receives accessible focus and scrolls into view; field-level errors do not cause global scrolling.</x:v>
+      </x:c>
+      <x:c r="H356" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="I356" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="J356" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K356" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L356" t="str">
+        <x:v>Blocking</x:v>
+      </x:c>
+      <x:c r="M356" t="str">
+        <x:v>L99-L115</x:v>
+      </x:c>
+      <x:c r="N356" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="O356" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P356" t="str">
+        <x:v>Automated local Sprint 3.1 regression PASS — 2026-09-16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="357">
+      <x:c r="A357" t="str">
+        <x:v>NOTIF-001</x:v>
+      </x:c>
+      <x:c r="B357" t="str">
+        <x:v>Notifications</x:v>
+      </x:c>
+      <x:c r="C357" t="str">
+        <x:v>In-app account notifications</x:v>
+      </x:c>
+      <x:c r="D357" t="str">
+        <x:v>Notification visibility, RLS and read state are owner-scoped</x:v>
+      </x:c>
+      <x:c r="E357" t="str">
+        <x:v>Two authenticated owners and supported lifecycle events exist.</x:v>
+      </x:c>
+      <x:c r="F357" t="str">
+        <x:v>Read notifications as each owner and anonymous; mark one notification read.</x:v>
+      </x:c>
+      <x:c r="G357" t="str">
+        <x:v>Each owner sees only their newest-first notifications; anonymous sees none; read state changes without mutable event/ownership metadata.</x:v>
+      </x:c>
+      <x:c r="H357" t="str">
+        <x:v>Particular / Store Owner</x:v>
+      </x:c>
+      <x:c r="I357" t="str">
+        <x:v>DB/Integration</x:v>
+      </x:c>
+      <x:c r="J357" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K357" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L357" t="str">
+        <x:v>Blocking</x:v>
+      </x:c>
+      <x:c r="M357" t="str">
+        <x:v>L254-L258</x:v>
+      </x:c>
+      <x:c r="N357" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="O357" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P357" t="str">
+        <x:v>Automated local Sprint 3.1 regression PASS — 2026-09-16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="358">
+      <x:c r="A358" t="str">
+        <x:v>NOTIF-002</x:v>
+      </x:c>
+      <x:c r="B358" t="str">
+        <x:v>Notifications</x:v>
+      </x:c>
+      <x:c r="C358" t="str">
+        <x:v>In-app account notifications</x:v>
+      </x:c>
+      <x:c r="D358" t="str">
+        <x:v>Revision rejection notification leads to its reason</x:v>
+      </x:c>
+      <x:c r="E358" t="str">
+        <x:v>Admin rejects an amended listing revision with a reason.</x:v>
+      </x:c>
+      <x:c r="F358" t="str">
+        <x:v>Open the owner notification and follow its target.</x:v>
+      </x:c>
+      <x:c r="G358" t="str">
+        <x:v>A typed rejection notice links to the owner's listing area where the rejection reason is reachable.</x:v>
+      </x:c>
+      <x:c r="H358" t="str">
+        <x:v>Particular / Store Owner</x:v>
+      </x:c>
+      <x:c r="I358" t="str">
+        <x:v>Integration</x:v>
+      </x:c>
+      <x:c r="J358" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K358" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L358" t="str">
+        <x:v>Blocking</x:v>
+      </x:c>
+      <x:c r="M358" t="str">
+        <x:v>L254-L258</x:v>
+      </x:c>
+      <x:c r="N358" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="O358" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P358" t="str">
+        <x:v>Automated local Sprint 3.1 regression PASS — 2026-09-16</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="O2:O350">
@@ -17411,7 +17875,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra74909d83f4d43f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ef17402a21741c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17461,7 +17925,7 @@
         <x:v>Total test cases</x:v>
       </x:c>
       <x:c r="B4" s="12" t="n">
-        <x:v>349</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="D4" s="12" t="str">
         <x:v>Public Marketplace</x:v>
@@ -17480,8 +17944,8 @@
         <x:v>P0 cases</x:v>
       </x:c>
       <x:c r="B5" s="12" t="n">
-        <x:f>COUNTIF('Acceptance Matrix'!K2:K350,"P0")</x:f>
-        <x:v>224</x:v>
+        <x:f>COUNTIF('Acceptance Matrix'!K2:K358,"P0")</x:f>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
         <x:v>Accounts &amp; Authentication</x:v>
@@ -17500,19 +17964,19 @@
         <x:v>Blocking cases</x:v>
       </x:c>
       <x:c r="B6" s="12" t="n">
-        <x:f>COUNTIF('Acceptance Matrix'!L2:L350,"Blocking")</x:f>
-        <x:v>341</x:v>
+        <x:f>COUNTIF('Acceptance Matrix'!L2:L358,"Blocking")</x:f>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
         <x:v>Listings</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
         <x:f>COUNTIF('Acceptance Matrix'!B:B,D6)</x:f>
-        <x:v>69</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="F6" s="12" t="n">
         <x:f>COUNTIFS('Acceptance Matrix'!B:B,D6,'Acceptance Matrix'!K:K,"P0")</x:f>
-        <x:v>47</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -17520,8 +17984,8 @@
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="B7" s="12" t="n">
-        <x:f>COUNTIF('Acceptance Matrix'!J2:J350,"Automated")</x:f>
-        <x:v>299</x:v>
+        <x:f>COUNTIF('Acceptance Matrix'!J2:J358,"Automated")</x:f>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
         <x:v>Security &amp; Ownership</x:v>
@@ -17540,7 +18004,7 @@
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="B8" s="12" t="n">
-        <x:f>COUNTIF('Acceptance Matrix'!J2:J350,"Manual")</x:f>
+        <x:f>COUNTIF('Acceptance Matrix'!J2:J358,"Manual")</x:f>
         <x:v>23</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
@@ -17548,7 +18012,7 @@
       </x:c>
       <x:c r="E8" s="12" t="n">
         <x:f>COUNTIF('Acceptance Matrix'!B:B,D8)</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F8" s="12" t="n">
         <x:f>COUNTIFS('Acceptance Matrix'!B:B,D8,'Acceptance Matrix'!K:K,"P0")</x:f>
@@ -17560,7 +18024,7 @@
         <x:v>Both</x:v>
       </x:c>
       <x:c r="B9" s="12" t="n">
-        <x:f>COUNTIF('Acceptance Matrix'!J2:J350,"Both")</x:f>
+        <x:f>COUNTIF('Acceptance Matrix'!J2:J358,"Both")</x:f>
         <x:v>27</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
@@ -17580,15 +18044,15 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="B10" s="12" t="n">
-        <x:f>COUNTIF('Acceptance Matrix'!O2:O350,"Pass")</x:f>
-        <x:v>81</x:v>
+        <x:f>COUNTIF('Acceptance Matrix'!O2:O358,"Pass")</x:f>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
         <x:v>Stores</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
         <x:f>COUNTIF('Acceptance Matrix'!B:B,D10)</x:f>
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F10" s="12" t="n">
         <x:f>COUNTIFS('Acceptance Matrix'!B:B,D10,'Acceptance Matrix'!K:K,"P0")</x:f>
@@ -17600,8 +18064,8 @@
         <x:v>Failed</x:v>
       </x:c>
       <x:c r="B11" s="12" t="n">
-        <x:f>COUNTIF('Acceptance Matrix'!O2:O350,"Fail")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF('Acceptance Matrix'!O2:O358,"Fail")</x:f>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
         <x:v>Store Dashboard</x:v>
@@ -17699,11 +18163,11 @@
       </x:c>
       <x:c r="E18" s="12" t="n">
         <x:f>COUNTIF('Acceptance Matrix'!B:B,D18)</x:f>
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F18" s="12" t="n">
         <x:f>COUNTIFS('Acceptance Matrix'!B:B,D18,'Acceptance Matrix'!K:K,"P0")</x:f>
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -17948,7 +18412,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99960cbd21274bf4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5c85e35058249b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18237,10 +18701,10 @@
         <x:v>L254-L258</x:v>
       </x:c>
       <x:c r="C20" s="12" t="str">
-        <x:v>MAIL</x:v>
+        <x:v>MAIL, NOTIF</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
-        <x:v>Centralized marketplace emails</x:v>
+        <x:v>Marketplace email infrastructure plus in-app account lifecycle notifications</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -18288,7 +18752,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R068000dbfd654911"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c7d2bb14a9b4d09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>